<commit_message>
amend state and federal scripts
</commit_message>
<xml_diff>
--- a/viz/data/cand_lists/2026_candidates_nonmatch.xlsx
+++ b/viz/data/cand_lists/2026_candidates_nonmatch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannahbensen/code/maine-monitor-campaign-finance/viz/data/cand_lists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D0BB2A-FF8A-434F-9671-5ACDE93333BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC8B0C4-B2B2-AB4A-B66A-75D3B36BC7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1760" yWindow="1000" windowWidth="27640" windowHeight="16860" xr2:uid="{41A728EB-2F27-7349-9880-2AB0051182C6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>filer_name</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Sheriff</t>
   </si>
   <si>
-    <t>House</t>
-  </si>
-  <si>
     <t>Republican</t>
   </si>
   <si>
@@ -111,6 +108,12 @@
   </si>
   <si>
     <t>John E. Ducharme, III</t>
+  </si>
+  <si>
+    <t>Representative</t>
+  </si>
+  <si>
+    <t>list</t>
   </si>
 </sst>
 </file>
@@ -504,14 +507,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA3363DC-5E83-234C-8C42-67D7AC7B31A7}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -524,163 +528,205 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C5" s="2">
         <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2">
         <v>87</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C9" s="2">
         <v>16</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2">
         <v>143</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="E11">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C12" s="2">
         <v>133</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="E12">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="C14" s="2">
         <v>71</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="E14">
+        <v>2024</v>
       </c>
     </row>
   </sheetData>

</xml_diff>